<commit_message>
updated rtm and execution summary
</commit_message>
<xml_diff>
--- a/OpenCart-RTM.xlsx
+++ b/OpenCart-RTM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/15d74eb5e75247de/Desktop/SQA_Projects/ManualTesting_OpenCart/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{0D1469AA-0D30-4C44-AB68-52A751D297CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D411C23A-BB72-4921-89AF-7E6EA4D6ABB5}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{0D1469AA-0D30-4C44-AB68-52A751D297CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D584D275-6DD2-45DF-90F8-28638B062E6D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{16F5F956-8860-4C89-91E7-5AB6E740AB8D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="115">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Coverage Status</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>TS_001</t>
   </si>
   <si>
@@ -180,9 +177,6 @@
     <t>Validate My Account functionality</t>
   </si>
   <si>
-    <t>TC_023</t>
-  </si>
-  <si>
     <t>TS_014</t>
   </si>
   <si>
@@ -291,9 +285,6 @@
     <t>Validate working of Affiliate functionality</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>Not Covered</t>
   </si>
   <si>
@@ -337,6 +328,48 @@
   </si>
   <si>
     <t>Validate the complete Application functionality for different currencies</t>
+  </si>
+  <si>
+    <t>TC Count</t>
+  </si>
+  <si>
+    <t>Execution Result</t>
+  </si>
+  <si>
+    <t>Defect ID</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Not covered</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Not Executed</t>
+  </si>
+  <si>
+    <t>BUG-001</t>
+  </si>
+  <si>
+    <t>BUG-002</t>
+  </si>
+  <si>
+    <t>BUG-003</t>
+  </si>
+  <si>
+    <t>BUG-004</t>
+  </si>
+  <si>
+    <t>BUG-005</t>
+  </si>
+  <si>
+    <t>No test case currently mapped to this scenario</t>
   </si>
 </sst>
 </file>
@@ -352,7 +385,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -367,6 +400,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -398,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -407,6 +452,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -721,18 +772,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5BC7EC-1EF0-4481-9682-346DF0356716}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
-    <col min="7" max="7" width="48.28515625" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="9" width="18.140625" customWidth="1"/>
+    <col min="10" max="10" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -746,679 +798,922 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="1">
+        <v>2</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="90" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="G5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1">
+        <v>2</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="G6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1">
+        <v>2</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="G7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="1">
+        <v>2</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="G8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="1"/>
-    </row>
-    <row r="9" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="1">
+        <v>2</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="G9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" ht="90" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="G10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="1"/>
-    </row>
-    <row r="11" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="1">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="G11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" ht="90" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="1">
+        <v>2</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="G13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E14" s="1" t="s">
+      <c r="B15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" ht="150" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="G15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="B16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="D16" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="G16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E16" s="1" t="s">
+      <c r="B17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="1"/>
-    </row>
-    <row r="17" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="D17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="1" t="s">
+      <c r="G17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="1"/>
-    </row>
-    <row r="18" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="D18" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="1" t="s">
+      <c r="G18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="B19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="1"/>
-    </row>
-    <row r="19" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="D19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="1" t="s">
+      <c r="G19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="B20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="D20" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="1">
+        <v>1</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="G20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="D21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E21" s="1" t="s">
+      <c r="B22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="D22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E22" s="1" t="s">
+      <c r="B23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="1"/>
-    </row>
-    <row r="23" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="D23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E23" s="1">
+        <v>1</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="G23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E23" s="1" t="s">
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="1"/>
-    </row>
-    <row r="24" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="D24" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="1">
+        <v>1</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="G24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E24" s="1" t="s">
+      <c r="B25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="1"/>
-    </row>
-    <row r="25" spans="1:7" ht="150" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="D25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E25" s="1">
+        <v>1</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="G25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+    </row>
+    <row r="26" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E25" s="1" t="s">
+      <c r="B26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="1"/>
-    </row>
-    <row r="26" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="D26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="H26" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I26" s="5"/>
+      <c r="J26" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26" s="1" t="s">
+    </row>
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="B27" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="D27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="1">
+        <v>1</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="G27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="1" t="s">
+      <c r="B28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="1" t="s">
+      <c r="D28" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="1">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I28" s="5"/>
+      <c r="J28" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G27" s="1"/>
-    </row>
-    <row r="28" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="B29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="D29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" s="1">
+        <v>0</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I29" s="5"/>
+      <c r="J29" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="D30" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+      <c r="B31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C30" s="1" t="s">
+      <c r="D31" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I31" s="5"/>
+      <c r="J31" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="150" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+      <c r="B32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="165" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="D32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>90</v>
+        <v>20</v>
+      </c>
+      <c r="E32" s="1">
+        <v>0</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I32" s="5"/>
+      <c r="J32" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1" xr:uid="{E0760C54-DB57-4FF5-84F3-B9D13B6FABC0}">
+      <formula1>"P0, P1, P2, P3, P4"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>